<commit_message>
feat(modeling): hoan thanh tien xu ly dac trung A06, mo hinh phan cum K-Means/GMM A07, chon k=4 A08 va xuat olist_clustered.parquet
</commit_message>
<xml_diff>
--- a/Phan_cong_nhiem_vu_Olist.xlsx
+++ b/Phan_cong_nhiem_vu_Olist.xlsx
@@ -1086,7 +1086,7 @@
       </c>
       <c r="L10" s="11" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="M10" s="5" t="n"/>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="L11" s="11" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="M11" s="5" t="n"/>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="L12" s="11" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="M12" s="5" t="n"/>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="L20" s="11" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="M20" s="5" t="n"/>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="L21" s="11" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="M21" s="5" t="n"/>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="L22" s="11" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="M22" s="5" t="n"/>
@@ -1804,7 +1804,7 @@
       </c>
       <c r="L23" s="11" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="M23" s="5" t="n"/>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="L24" s="11" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="M24" s="5" t="n"/>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="L25" s="11" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="M25" s="5" t="n"/>
@@ -3252,7 +3252,7 @@
       </c>
       <c r="L49" s="11" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="M49" s="5" t="n"/>
@@ -3306,7 +3306,7 @@
       </c>
       <c r="L50" s="11" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="M50" s="5" t="n"/>

</xml_diff>